<commit_message>
Rename 'Professor's Notes' persona/label -> 'Scenario Rationale' across the skill
Drops the Gemini-Gems-origin HBS-finance-professor persona and the 'Professor's Strategic Notes' label everywhere in the live skill: stage4_modeler.md (persona line + section), README.md (Modeler persona -> 'Valuation analyst'; tab label), the .gs reference models (buildProfessorNotes->buildScenarioRationale, header strings), evals grader criterion. Regenerated example/GOOGL_Demo_Integrated_Financials.xlsx (now 'SCENARIO RATIONALE — {SCENARIO}') and rebuilt bav-pipeline-plugin.zip. Archived legacy/ Gem instructions left untouched as the historical record the README Lineage section points to. Verified: zero 'professor' in all live files, workbooks, and the shipped zip.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example/GOOGL_Demo_Integrated_Financials.xlsx
+++ b/example/GOOGL_Demo_Integrated_Financials.xlsx
@@ -7418,7 +7418,7 @@
     <row r="83">
       <c r="A83" s="76" t="inlineStr">
         <is>
-          <t>PROFESSOR'S STRATEGIC NOTES — BULL</t>
+          <t>SCENARIO RATIONALE — BULL</t>
         </is>
       </c>
       <c r="B83" s="99" t="n"/>
@@ -32940,7 +32940,7 @@
     <row r="83">
       <c r="A83" s="76" t="inlineStr">
         <is>
-          <t>PROFESSOR'S STRATEGIC NOTES — BEAR</t>
+          <t>SCENARIO RATIONALE — BEAR</t>
         </is>
       </c>
       <c r="B83" s="99" t="n"/>
@@ -36354,7 +36354,7 @@
     <row r="83">
       <c r="A83" s="76" t="inlineStr">
         <is>
-          <t>PROFESSOR'S STRATEGIC NOTES — BASE</t>
+          <t>SCENARIO RATIONALE — BASE</t>
         </is>
       </c>
       <c r="B83" s="99" t="n"/>

</xml_diff>

<commit_message>
GOOGL demo: use the real coverage assumptions (numbers real, scenario reasoning withheld)
The demo now mirrors the actual GOOGL spreadsheet's model inputs (real forecast vectors, betas, terminal growth, probabilities 15/50/35, price) instead of generic illustrative ones. Only the written scenario reasoning is withheld (placeholder) and the 'what must be true' rationalization stories stay out (mechanical ICC block kept). README example section corrected (was 'deliberately illustrative'); plugin.json -> 2.1.1; zip rebuilt. Demo raw-XML leak-scanned clean (no professor / research strings / other-ticker refs).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example/GOOGL_Demo_Integrated_Financials.xlsx
+++ b/example/GOOGL_Demo_Integrated_Financials.xlsx
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEMO WORKBOOK: financial data as filed with the SEC (real); model inputs ILLUSTRATIVE ONLY — not analysis, not advice.</t>
+          <t>DEMO WORKBOOK: as-filed SEC financials (real) + the analyst's actual GOOGL model assumptions; scenario reasoning withheld. Illustrates the system; not investment advice.</t>
         </is>
       </c>
     </row>
@@ -4603,34 +4603,34 @@
         <v/>
       </c>
       <c r="L11" s="29" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="M11" s="29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N11" s="29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O11" s="29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="P11" s="29" t="n">
         <v>0.2</v>
       </c>
-      <c r="M11" s="29" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="N11" s="29" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="O11" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="P11" s="29" t="n">
+      <c r="Q11" s="29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R11" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S11" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T11" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q11" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="R11" s="29" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="S11" s="29" t="n">
+      <c r="U11" s="29" t="n">
         <v>0.06</v>
-      </c>
-      <c r="T11" s="29" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="U11" s="29" t="n">
-        <v>0.04</v>
       </c>
       <c r="W11" s="1">
         <f>AVERAGE(C11:K11)</f>
@@ -4684,34 +4684,34 @@
         <v/>
       </c>
       <c r="L12" s="29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M12" s="29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="N12" s="29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O12" s="29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P12" s="29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="Q12" s="29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="R12" s="29" t="n">
         <v>0.32</v>
       </c>
-      <c r="M12" s="29" t="n">
-        <v>0.315</v>
-      </c>
-      <c r="N12" s="29" t="n">
+      <c r="S12" s="29" t="n">
         <v>0.31</v>
       </c>
-      <c r="O12" s="29" t="n">
-        <v>0.305</v>
-      </c>
-      <c r="P12" s="29" t="n">
+      <c r="T12" s="29" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="U12" s="29" t="n">
         <v>0.3</v>
-      </c>
-      <c r="Q12" s="29" t="n">
-        <v>0.295</v>
-      </c>
-      <c r="R12" s="29" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="S12" s="29" t="n">
-        <v>0.285</v>
-      </c>
-      <c r="T12" s="29" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="U12" s="29" t="n">
-        <v>0.28</v>
       </c>
       <c r="W12" s="1">
         <f>AVERAGE(C12:K12)</f>
@@ -4766,35 +4766,36 @@
         <f>K21/K31</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="n">
-        <v>0.02</v>
+      <c r="L14" s="30">
+        <f>L21/L31</f>
+        <v/>
       </c>
       <c r="M14" s="31" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="N14" s="31" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="O14" s="31" t="n">
-        <v>0.035</v>
+        <v>0</v>
       </c>
       <c r="P14" s="31" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="31" t="n">
-        <v>0.045</v>
+        <v>0</v>
       </c>
       <c r="R14" s="31" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="S14" s="31" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="T14" s="31" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="U14" s="31" t="n">
-        <v>0.065</v>
+        <v>0</v>
       </c>
       <c r="W14" s="2">
         <f>AVERAGE(C14:K14)</f>
@@ -4848,35 +4849,36 @@
         <f>K22/K31</f>
         <v/>
       </c>
-      <c r="L15" s="30" t="n">
-        <v>0.5</v>
+      <c r="L15" s="30">
+        <f>L22/L31</f>
+        <v/>
       </c>
       <c r="M15" s="31" t="n">
-        <v>0.55</v>
+        <v>0.9821</v>
       </c>
       <c r="N15" s="31" t="n">
-        <v>0.6</v>
+        <v>1.0321</v>
       </c>
       <c r="O15" s="31" t="n">
-        <v>0.65</v>
+        <v>1.0821</v>
       </c>
       <c r="P15" s="31" t="n">
-        <v>0.7</v>
+        <v>1.1221</v>
       </c>
       <c r="Q15" s="31" t="n">
-        <v>0.75</v>
+        <v>1.1621</v>
       </c>
       <c r="R15" s="31" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="S15" s="31" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="T15" s="31" t="n">
         <v>0.9</v>
       </c>
       <c r="U15" s="31" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="W15" s="2">
         <f>AVERAGE(C15:K15)</f>
@@ -7445,7 +7447,7 @@
     <row r="84">
       <c r="A84" s="99" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE BULL — generic durable-growth inputs for demonstration. Not analysis.</t>
+          <t>Scenario reasoning is withheld from the public demo. The blue model inputs above are the actual GOOGL coverage assumptions; the written rationale behind them is kept private. Not investment advice.</t>
         </is>
       </c>
       <c r="B84" s="99" t="n"/>
@@ -7796,7 +7798,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Probability-Weighted Residual Income Valuation — ILLUSTRATIVE inputs (see model tabs); not analysis</t>
+          <t>Probability-Weighted Residual Income Valuation — GOOGL coverage build (as-analyzed inputs; scenario reasoning withheld). Not investment advice.</t>
         </is>
       </c>
     </row>
@@ -7835,13 +7837,13 @@
         </is>
       </c>
       <c r="B5" s="33" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="C5" s="33" t="n">
         <v>0.5</v>
       </c>
       <c r="D5" s="33" t="n">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="6"/>
@@ -9020,7 +9022,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Live ICC: the discount rate at which each scenario's IVPS equals the price in B5. Reactive — recomputes when the price or any model input changes. Model inputs ILLUSTRATIVE; not analysis.</t>
+          <t>Live ICC: the discount rate at which each scenario's IVPS equals the price in B5. Reactive — recomputes when the price or any model input changes. GOOGL coverage build; not investment advice.</t>
         </is>
       </c>
     </row>
@@ -30125,34 +30127,34 @@
         <v/>
       </c>
       <c r="L11" s="29" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M11" s="29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N11" s="29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O11" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P11" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q11" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="M11" s="29" t="n">
+      <c r="R11" s="29" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S11" s="29" t="n">
         <v>0.08</v>
       </c>
-      <c r="N11" s="29" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="O11" s="29" t="n">
+      <c r="T11" s="29" t="n">
         <v>0.05</v>
       </c>
-      <c r="P11" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="Q11" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="R11" s="29" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="S11" s="29" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="T11" s="29" t="n">
-        <v>0.03</v>
-      </c>
       <c r="U11" s="29" t="n">
-        <v>0.03</v>
+        <v>0.035</v>
       </c>
       <c r="W11" s="1">
         <f>AVERAGE(C11:K11)</f>
@@ -30206,34 +30208,34 @@
         <v/>
       </c>
       <c r="L12" s="29" t="n">
-        <v>0.24</v>
+        <v>0.32</v>
       </c>
       <c r="M12" s="29" t="n">
-        <v>0.235</v>
+        <v>0.31</v>
       </c>
       <c r="N12" s="29" t="n">
-        <v>0.23</v>
+        <v>0.3</v>
       </c>
       <c r="O12" s="29" t="n">
-        <v>0.225</v>
+        <v>0.3</v>
       </c>
       <c r="P12" s="29" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="Q12" s="29" t="n">
-        <v>0.215</v>
+        <v>0.29</v>
       </c>
       <c r="R12" s="29" t="n">
-        <v>0.21</v>
+        <v>0.28</v>
       </c>
       <c r="S12" s="29" t="n">
-        <v>0.205</v>
+        <v>0.28</v>
       </c>
       <c r="T12" s="29" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
       </c>
       <c r="U12" s="29" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="W12" s="1">
         <f>AVERAGE(C12:K12)</f>
@@ -30288,35 +30290,36 @@
         <f>K21/K31</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="n">
-        <v>0.02</v>
+      <c r="L14" s="30">
+        <f>L21/L31</f>
+        <v/>
       </c>
       <c r="M14" s="31" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="N14" s="31" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="O14" s="31" t="n">
-        <v>0.035</v>
+        <v>0</v>
       </c>
       <c r="P14" s="31" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="31" t="n">
-        <v>0.045</v>
+        <v>0</v>
       </c>
       <c r="R14" s="31" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="S14" s="31" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="T14" s="31" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="U14" s="31" t="n">
-        <v>0.065</v>
+        <v>0</v>
       </c>
       <c r="W14" s="2">
         <f>AVERAGE(C14:K14)</f>
@@ -30370,35 +30373,36 @@
         <f>K22/K31</f>
         <v/>
       </c>
-      <c r="L15" s="30" t="n">
-        <v>0.5</v>
+      <c r="L15" s="30">
+        <f>L22/L31</f>
+        <v/>
       </c>
       <c r="M15" s="31" t="n">
-        <v>0.55</v>
+        <v>1.0221</v>
       </c>
       <c r="N15" s="31" t="n">
-        <v>0.6</v>
+        <v>1.1221</v>
       </c>
       <c r="O15" s="31" t="n">
-        <v>0.65</v>
+        <v>1.2021</v>
       </c>
       <c r="P15" s="31" t="n">
-        <v>0.7</v>
+        <v>1.2821</v>
       </c>
       <c r="Q15" s="31" t="n">
-        <v>0.75</v>
+        <v>1.3521</v>
       </c>
       <c r="R15" s="31" t="n">
-        <v>0.8</v>
+        <v>1.4121</v>
       </c>
       <c r="S15" s="31" t="n">
-        <v>0.85</v>
+        <v>1.4621</v>
       </c>
       <c r="T15" s="31" t="n">
-        <v>0.9</v>
+        <v>1.5121</v>
       </c>
       <c r="U15" s="31" t="n">
-        <v>0.95</v>
+        <v>1.5521</v>
       </c>
       <c r="W15" s="2">
         <f>AVERAGE(C15:K15)</f>
@@ -32967,7 +32971,7 @@
     <row r="84">
       <c r="A84" s="99" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE BEAR — generic deceleration-and-compression inputs for demonstration. Not analysis. Run /bav-pipeline to build scenarios from an actual strategy report.</t>
+          <t>Scenario reasoning is withheld from the public demo. The blue model inputs above are the actual GOOGL coverage assumptions; the written rationale behind them is kept private. Not investment advice.</t>
         </is>
       </c>
       <c r="B84" s="99" t="n"/>
@@ -33322,7 +33326,7 @@
         </is>
       </c>
       <c r="B2" s="26" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="3">
@@ -33539,34 +33543,34 @@
         <v/>
       </c>
       <c r="L11" s="29" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="M11" s="29" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="N11" s="29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O11" s="29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P11" s="29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q11" s="29" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="R11" s="29" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="S11" s="29" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="T11" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="O11" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="P11" s="29" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="Q11" s="29" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="R11" s="29" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="S11" s="29" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="T11" s="29" t="n">
+      <c r="U11" s="29" t="n">
         <v>0.04</v>
-      </c>
-      <c r="U11" s="29" t="n">
-        <v>0.035</v>
       </c>
       <c r="W11" s="1">
         <f>AVERAGE(C11:K11)</f>
@@ -33620,34 +33624,34 @@
         <v/>
       </c>
       <c r="L12" s="29" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="M12" s="29" t="n">
-        <v>0.275</v>
+        <v>0.32</v>
       </c>
       <c r="N12" s="29" t="n">
-        <v>0.27</v>
+        <v>0.32</v>
       </c>
       <c r="O12" s="29" t="n">
-        <v>0.265</v>
+        <v>0.32</v>
       </c>
       <c r="P12" s="29" t="n">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
       <c r="Q12" s="29" t="n">
-        <v>0.255</v>
+        <v>0.32</v>
       </c>
       <c r="R12" s="29" t="n">
-        <v>0.25</v>
+        <v>0.32</v>
       </c>
       <c r="S12" s="29" t="n">
-        <v>0.245</v>
+        <v>0.31</v>
       </c>
       <c r="T12" s="29" t="n">
-        <v>0.24</v>
+        <v>0.31</v>
       </c>
       <c r="U12" s="29" t="n">
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="W12" s="1">
         <f>AVERAGE(C12:K12)</f>
@@ -33702,35 +33706,36 @@
         <f>K21/K31</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="n">
-        <v>0.02</v>
+      <c r="L14" s="30">
+        <f>L21/L31</f>
+        <v/>
       </c>
       <c r="M14" s="31" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="N14" s="31" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="O14" s="31" t="n">
-        <v>0.035</v>
+        <v>0</v>
       </c>
       <c r="P14" s="31" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="31" t="n">
-        <v>0.045</v>
+        <v>0</v>
       </c>
       <c r="R14" s="31" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="S14" s="31" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="T14" s="31" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="U14" s="31" t="n">
-        <v>0.065</v>
+        <v>0</v>
       </c>
       <c r="W14" s="2">
         <f>AVERAGE(C14:K14)</f>
@@ -33784,35 +33789,36 @@
         <f>K22/K31</f>
         <v/>
       </c>
-      <c r="L15" s="30" t="n">
-        <v>0.5</v>
+      <c r="L15" s="30">
+        <f>L22/L31</f>
+        <v/>
       </c>
       <c r="M15" s="31" t="n">
-        <v>0.55</v>
+        <v>0.9821</v>
       </c>
       <c r="N15" s="31" t="n">
-        <v>0.6</v>
+        <v>1.0321</v>
       </c>
       <c r="O15" s="31" t="n">
-        <v>0.65</v>
+        <v>1.0821</v>
       </c>
       <c r="P15" s="31" t="n">
-        <v>0.7</v>
+        <v>1.1221</v>
       </c>
       <c r="Q15" s="31" t="n">
-        <v>0.75</v>
+        <v>1.1621</v>
       </c>
       <c r="R15" s="31" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="S15" s="31" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="T15" s="31" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="U15" s="31" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="W15" s="2">
         <f>AVERAGE(C15:K15)</f>
@@ -36381,7 +36387,7 @@
     <row r="84">
       <c r="A84" s="99" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE BASE — generic moderate-fade inputs for demonstration. Not analysis.</t>
+          <t>Scenario reasoning is withheld from the public demo. The blue model inputs above are the actual GOOGL coverage assumptions; the written rationale behind them is kept private. Not investment advice.</t>
         </is>
       </c>
       <c r="B84" s="99" t="n"/>

</xml_diff>

<commit_message>
GOOGL demo: ship the full real coverage build (assumptions + reasoning); restore 'deliberately illustrative'
The demo is now a faithful copy of the real GOOGL spreadsheet — real inputs AND the per-scenario Scenario Rationale reasoning — with only the price-rationalization (valuation-rationale) tab held back (replaced by the mechanical Implied Cost of Capital tab). README example section restores the 'deliberately illustrative / not investment advice' framing (kept truthful — no false 'generic textbook vectors' claim). plugin.json -> 2.1.2; zip rebuilt. Demo raw-XML leak-scanned clean (no professor / protected-research strings / other-ticker refs).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example/GOOGL_Demo_Integrated_Financials.xlsx
+++ b/example/GOOGL_Demo_Integrated_Financials.xlsx
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEMO WORKBOOK: as-filed SEC financials (real) + the analyst's actual GOOGL model assumptions; scenario reasoning withheld. Illustrates the system; not investment advice.</t>
+          <t>DEMO WORKBOOK — deliberately illustrative: a complete, real GOOGL coverage build (as-filed SEC financials + the analyst's actual model assumptions and reasoning) shown to demonstrate the system. Not investment advice.</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
     <row r="83">
       <c r="A83" s="76" t="inlineStr">
         <is>
-          <t>SCENARIO RATIONALE — BULL</t>
+          <t>SCENARIO RATIONALE — BULL CASE</t>
         </is>
       </c>
       <c r="B83" s="99" t="n"/>
@@ -7445,11 +7445,7 @@
       <c r="U83" s="99" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="99" t="inlineStr">
-        <is>
-          <t>Scenario reasoning is withheld from the public demo. The blue model inputs above are the actual GOOGL coverage assumptions; the written rationale behind them is kept private. Not investment advice.</t>
-        </is>
-      </c>
+      <c r="A84" s="99" t="n"/>
       <c r="B84" s="99" t="n"/>
       <c r="C84" s="99" t="n"/>
       <c r="D84" s="99" t="n"/>
@@ -7472,7 +7468,11 @@
       <c r="U84" s="99" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="76" t="n"/>
+      <c r="A85" s="76" t="inlineStr">
+        <is>
+          <t>Growth Assumption Rationale:</t>
+        </is>
+      </c>
       <c r="B85" s="99" t="n"/>
       <c r="C85" s="99" t="n"/>
       <c r="D85" s="99" t="n"/>
@@ -7495,6 +7495,11 @@
       <c r="U85" s="99" t="n"/>
     </row>
     <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>AI supercharges Search monetization (higher RPQ, new ad formats). Cloud accelerates to become #2 behind AWS at 30%+ margins. Gemini ecosystem drives new revenue streams. Waymo begins meaningful revenue contribution.</t>
+        </is>
+      </c>
       <c r="B86" s="99" t="n"/>
       <c r="C86" s="99" t="n"/>
       <c r="D86" s="99" t="n"/>
@@ -7540,7 +7545,11 @@
       <c r="U87" s="99" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="76" t="n"/>
+      <c r="A88" s="76" t="inlineStr">
+        <is>
+          <t>Margin &amp; Moat Assessment:</t>
+        </is>
+      </c>
       <c r="B88" s="99" t="n"/>
       <c r="C88" s="99" t="n"/>
       <c r="D88" s="99" t="n"/>
@@ -7563,6 +7572,11 @@
       <c r="U88" s="99" t="n"/>
     </row>
     <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Full-stack AI moat proves durable. Operating margins expand near-term as Cloud reaches scale economies. CapEx investments generate strong ROIC through proprietary TPU advantages and data flywheel effects.</t>
+        </is>
+      </c>
       <c r="B89" s="99" t="n"/>
       <c r="C89" s="99" t="n"/>
       <c r="D89" s="99" t="n"/>
@@ -7608,7 +7622,11 @@
       <c r="U90" s="99" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="76" t="n"/>
+      <c r="A91" s="76" t="inlineStr">
+        <is>
+          <t>Key Risks to Monitor:</t>
+        </is>
+      </c>
       <c r="B91" s="99" t="n"/>
       <c r="C91" s="99" t="n"/>
       <c r="D91" s="99" t="n"/>
@@ -7631,6 +7649,11 @@
       <c r="U91" s="99" t="n"/>
     </row>
     <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Antitrust outcome more benign than feared. AI investment cycle pays off faster than expected. Risk of overpaying for growth if AI hype deflates.</t>
+        </is>
+      </c>
       <c r="B92" s="99" t="n"/>
       <c r="C92" s="99" t="n"/>
       <c r="D92" s="99" t="n"/>
@@ -7676,7 +7699,11 @@
       <c r="U93" s="99" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="76" t="n"/>
+      <c r="A94" s="76" t="inlineStr">
+        <is>
+          <t>Valuation Context:</t>
+        </is>
+      </c>
       <c r="B94" s="99" t="n"/>
       <c r="C94" s="99" t="n"/>
       <c r="D94" s="99" t="n"/>
@@ -7699,6 +7726,11 @@
       <c r="U94" s="99" t="n"/>
     </row>
     <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Bull case reflects Alphabet as the preeminent AI platform company, successfully monetizing its unique vertical integration across hardware, models, applications, and distribution.</t>
+        </is>
+      </c>
       <c r="B95" s="99" t="n"/>
       <c r="C95" s="99" t="n"/>
       <c r="D95" s="99" t="n"/>
@@ -7798,7 +7830,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Probability-Weighted Residual Income Valuation — GOOGL coverage build (as-analyzed inputs; scenario reasoning withheld). Not investment advice.</t>
+          <t>Probability-Weighted Residual Income Valuation — deliberately illustrative demo (a real GOOGL coverage build). Not investment advice.</t>
         </is>
       </c>
     </row>
@@ -9022,7 +9054,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Live ICC: the discount rate at which each scenario's IVPS equals the price in B5. Reactive — recomputes when the price or any model input changes. GOOGL coverage build; not investment advice.</t>
+          <t>Live ICC: the discount rate at which each scenario's IVPS equals the price in B5. Reactive — recomputes when the price or any model input changes. Deliberately illustrative demo; not investment advice.</t>
         </is>
       </c>
     </row>
@@ -32944,7 +32976,7 @@
     <row r="83">
       <c r="A83" s="76" t="inlineStr">
         <is>
-          <t>SCENARIO RATIONALE — BEAR</t>
+          <t>SCENARIO RATIONALE — BEAR CASE</t>
         </is>
       </c>
       <c r="B83" s="99" t="n"/>
@@ -32969,11 +33001,7 @@
       <c r="U83" s="99" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="99" t="inlineStr">
-        <is>
-          <t>Scenario reasoning is withheld from the public demo. The blue model inputs above are the actual GOOGL coverage assumptions; the written rationale behind them is kept private. Not investment advice.</t>
-        </is>
-      </c>
+      <c r="A84" s="99" t="n"/>
       <c r="B84" s="99" t="n"/>
       <c r="C84" s="99" t="n"/>
       <c r="D84" s="99" t="n"/>
@@ -32996,7 +33024,11 @@
       <c r="U84" s="99" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="76" t="n"/>
+      <c r="A85" s="76" t="inlineStr">
+        <is>
+          <t>Growth Assumption Rationale:</t>
+        </is>
+      </c>
       <c r="B85" s="99" t="n"/>
       <c r="C85" s="99" t="n"/>
       <c r="D85" s="99" t="n"/>
@@ -33019,6 +33051,11 @@
       <c r="U85" s="99" t="n"/>
     </row>
     <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>AI disrupts Search ad monetization; Cloud growth decelerates to &lt;20% as pricing pressure from AWS/Azure intensifies. Antitrust remedies (Chrome/AdX divestiture) structurally weaken ecosystem. Revenue growth trends toward GDP+inflation.</t>
+        </is>
+      </c>
       <c r="B86" s="99" t="n"/>
       <c r="C86" s="99" t="n"/>
       <c r="D86" s="99" t="n"/>
@@ -33064,7 +33101,11 @@
       <c r="U87" s="99" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="76" t="n"/>
+      <c r="A88" s="76" t="inlineStr">
+        <is>
+          <t>Margin &amp; Moat Assessment:</t>
+        </is>
+      </c>
       <c r="B88" s="99" t="n"/>
       <c r="C88" s="99" t="n"/>
       <c r="D88" s="99" t="n"/>
@@ -33087,6 +33128,11 @@
       <c r="U88" s="99" t="n"/>
     </row>
     <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Search share erodes to ~75% as AI alternatives gain traction. Cloud margins plateau at ~20%. Operating margin compresses toward 25% as massive CapEx ($175B+) fails to generate proportional returns.</t>
+        </is>
+      </c>
       <c r="B89" s="99" t="n"/>
       <c r="C89" s="99" t="n"/>
       <c r="D89" s="99" t="n"/>
@@ -33132,7 +33178,11 @@
       <c r="U90" s="99" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="76" t="n"/>
+      <c r="A91" s="76" t="inlineStr">
+        <is>
+          <t>Key Risks to Monitor:</t>
+        </is>
+      </c>
       <c r="B91" s="99" t="n"/>
       <c r="C91" s="99" t="n"/>
       <c r="D91" s="99" t="n"/>
@@ -33155,6 +33205,11 @@
       <c r="U91" s="99" t="n"/>
     </row>
     <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DOJ structural breakup, AI cannibalization of Search revenue, CapEx overcapacity, geopolitical chip supply disruption, regulatory fines accumulating globally.</t>
+        </is>
+      </c>
       <c r="B92" s="99" t="n"/>
       <c r="C92" s="99" t="n"/>
       <c r="D92" s="99" t="n"/>
@@ -33200,7 +33255,11 @@
       <c r="U93" s="99" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="76" t="n"/>
+      <c r="A94" s="76" t="inlineStr">
+        <is>
+          <t>Valuation Context:</t>
+        </is>
+      </c>
       <c r="B94" s="99" t="n"/>
       <c r="C94" s="99" t="n"/>
       <c r="D94" s="99" t="n"/>
@@ -33223,6 +33282,11 @@
       <c r="U94" s="99" t="n"/>
     </row>
     <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Bear case reflects a world where Alphabet becomes a regulated utility-like company with deteriorating competitive position and massive capital requirements.</t>
+        </is>
+      </c>
       <c r="B95" s="99" t="n"/>
       <c r="C95" s="99" t="n"/>
       <c r="D95" s="99" t="n"/>
@@ -33245,7 +33309,11 @@
       <c r="U95" s="99" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="74" t="n"/>
+      <c r="A96" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Company becomes way more capital intensive, and under intense competition, margins erode and sales growth from investments not as significant. </t>
+        </is>
+      </c>
       <c r="B96" s="99" t="n"/>
       <c r="C96" s="99" t="n"/>
       <c r="D96" s="99" t="n"/>
@@ -36360,7 +36428,7 @@
     <row r="83">
       <c r="A83" s="76" t="inlineStr">
         <is>
-          <t>SCENARIO RATIONALE — BASE</t>
+          <t>SCENARIO RATIONALE — BASE CASE</t>
         </is>
       </c>
       <c r="B83" s="99" t="n"/>
@@ -36385,11 +36453,7 @@
       <c r="U83" s="99" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="99" t="inlineStr">
-        <is>
-          <t>Scenario reasoning is withheld from the public demo. The blue model inputs above are the actual GOOGL coverage assumptions; the written rationale behind them is kept private. Not investment advice.</t>
-        </is>
-      </c>
+      <c r="A84" s="99" t="n"/>
       <c r="B84" s="99" t="n"/>
       <c r="C84" s="99" t="n"/>
       <c r="D84" s="99" t="n"/>
@@ -36412,7 +36476,11 @@
       <c r="U84" s="99" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="76" t="n"/>
+      <c r="A85" s="76" t="inlineStr">
+        <is>
+          <t>Growth Assumption Rationale:</t>
+        </is>
+      </c>
       <c r="B85" s="99" t="n"/>
       <c r="C85" s="99" t="n"/>
       <c r="D85" s="99" t="n"/>
@@ -36435,6 +36503,11 @@
       <c r="U85" s="99" t="n"/>
     </row>
     <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Search maintains dominance with AI Overviews enhancing engagement. Cloud sustains 20-25% growth through AI Vertex platform. YouTube crosses $60B+ annually. Revenue growth gradually decelerates as base expands past $500B.</t>
+        </is>
+      </c>
       <c r="B86" s="99" t="n"/>
       <c r="C86" s="99" t="n"/>
       <c r="D86" s="99" t="n"/>
@@ -36480,7 +36553,11 @@
       <c r="U87" s="99" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="76" t="n"/>
+      <c r="A88" s="76" t="inlineStr">
+        <is>
+          <t>Margin &amp; Moat Assessment:</t>
+        </is>
+      </c>
       <c r="B88" s="99" t="n"/>
       <c r="C88" s="99" t="n"/>
       <c r="D88" s="99" t="n"/>
@@ -36503,6 +36580,11 @@
       <c r="U88" s="99" t="n"/>
     </row>
     <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Full-stack advantage (Gemini + TPUs + Android/Chrome + Search data) provides durable moat. Operating margins stabilize ~27% near-term then compress modestly as CapEx normalizes. Antitrust results in behavioral remedies, not structural breakup.</t>
+        </is>
+      </c>
       <c r="B89" s="99" t="n"/>
       <c r="C89" s="99" t="n"/>
       <c r="D89" s="99" t="n"/>
@@ -36548,7 +36630,11 @@
       <c r="U90" s="99" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="76" t="n"/>
+      <c r="A91" s="76" t="inlineStr">
+        <is>
+          <t>Key Risks to Monitor:</t>
+        </is>
+      </c>
       <c r="B91" s="99" t="n"/>
       <c r="C91" s="99" t="n"/>
       <c r="D91" s="99" t="n"/>
@@ -36571,6 +36657,11 @@
       <c r="U91" s="99" t="n"/>
     </row>
     <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>AI competition from OpenAI/Meta intensifies, margin pressure from $175B+ annual CapEx, some Search cannibalization offset by Cloud growth, moderate regulatory drag.</t>
+        </is>
+      </c>
       <c r="B92" s="99" t="n"/>
       <c r="C92" s="99" t="n"/>
       <c r="D92" s="99" t="n"/>
@@ -36616,7 +36707,11 @@
       <c r="U93" s="99" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="76" t="n"/>
+      <c r="A94" s="76" t="inlineStr">
+        <is>
+          <t>Valuation Context:</t>
+        </is>
+      </c>
       <c r="B94" s="99" t="n"/>
       <c r="C94" s="99" t="n"/>
       <c r="D94" s="99" t="n"/>
@@ -36639,6 +36734,11 @@
       <c r="U94" s="99" t="n"/>
     </row>
     <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Base case reflects Alphabet as a dominant but maturing tech platform that successfully navigates the AI transition while returning capital aggressively through buybacks and dividends.</t>
+        </is>
+      </c>
       <c r="B95" s="99" t="n"/>
       <c r="C95" s="99" t="n"/>
       <c r="D95" s="99" t="n"/>
@@ -36661,7 +36761,11 @@
       <c r="U95" s="99" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="74" t="n"/>
+      <c r="A96" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Company bcomes more capital intensive, bringing down RNOA, but ultimately drives search (revenues) and increases margins. </t>
+        </is>
+      </c>
       <c r="B96" s="99" t="n"/>
       <c r="C96" s="99" t="n"/>
       <c r="D96" s="99" t="n"/>

</xml_diff>